<commit_message>
Version 2: houses play as one
- One (or two) secret Traitor houses, chosen eyes-closed
- Missions: every house answers every question on the floor, 3-2-1 lock-in, tutor marks wrong houses
- Round Table: per-house evidence; each house casts one vote, revealed one by one; tie = revote
- Night: poison (no vote at next Round Table) or dagger (murder; one per Traitor house)
- Ghost houses keep answering, never vote; Traitors win if they match the Faithful in votes
- Intro and host lines updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JwtKYzfmdJ9GJGzFpN9Now
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -508,7 +508,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>How many questions? Each round asks one per house. 5 houses x 4 rounds = 20, so 30+ means no repeats; 60+ is ideal.</t>
+          <t>How many questions? Each mission asks 3 (every house answers each). 4 rounds = 12 questions, so 20+ means no repeats; 40+ is ideal.</t>
         </is>
       </c>
     </row>
@@ -5955,7 +5955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6004,24 +6004,54 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pounds added to the prize pot for each right mission answer</t>
+          <t>Pounds added to the prize pot for each house that answers a mission question right</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Discussion minutes</t>
+          <t>Questions per mission</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="inlineStr">
+        <is>
+          <t>How many questions each mission has (every house answers each one)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Seconds per question</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Thinking time before houses lock in their answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Discussion minutes</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>Length of each Round Table discussion</t>
         </is>

</xml_diff>